<commit_message>
Reset canonical dataset to clean 9-10-1030 (drop test merge)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -886,11 +886,11 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to THLCH ~2026-09-11T23:00:00</t>
+          <t>Alongside, departs to THLCH ~2026-09-11T15:00:00</t>
         </is>
       </c>
       <c r="I7" s="3" t="n">
-        <v>46296.04166666666</v>
+        <v>46295.70833333334</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>46277.16666666666</v>
+        <v>46276.83333333334</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
@@ -6503,13 +6503,13 @@
         </is>
       </c>
       <c r="G97" s="3" t="n">
-        <v>46274.5</v>
+        <v>46274.16666666666</v>
       </c>
       <c r="H97" s="3" t="n">
-        <v>46274.54166666666</v>
+        <v>46274.20833333334</v>
       </c>
       <c r="I97" s="3" t="n">
-        <v>46275</v>
+        <v>46274.66666666666</v>
       </c>
     </row>
     <row r="98">
@@ -6544,13 +6544,13 @@
         </is>
       </c>
       <c r="G98" s="3" t="n">
-        <v>46275.08333333334</v>
+        <v>46274.75</v>
       </c>
       <c r="H98" s="3" t="n">
-        <v>46275.20833333334</v>
+        <v>46274.875</v>
       </c>
       <c r="I98" s="3" t="n">
-        <v>46276.95833333334</v>
+        <v>46276.625</v>
       </c>
     </row>
     <row r="99">
@@ -6585,13 +6585,13 @@
         </is>
       </c>
       <c r="G99" s="3" t="n">
-        <v>46275.08333333334</v>
+        <v>46274.75</v>
       </c>
       <c r="H99" s="3" t="n">
-        <v>46275.20833333334</v>
+        <v>46274.875</v>
       </c>
       <c r="I99" s="3" t="n">
-        <v>46276.95833333334</v>
+        <v>46276.625</v>
       </c>
     </row>
     <row r="100">
@@ -6626,13 +6626,13 @@
         </is>
       </c>
       <c r="G100" s="3" t="n">
-        <v>46277.16666666666</v>
+        <v>46276.83333333334</v>
       </c>
       <c r="H100" s="3" t="n">
-        <v>46277.20833333334</v>
+        <v>46276.875</v>
       </c>
       <c r="I100" s="3" t="n">
-        <v>46277.625</v>
+        <v>46277.29166666666</v>
       </c>
     </row>
     <row r="101">
@@ -6667,13 +6667,13 @@
         </is>
       </c>
       <c r="G101" s="3" t="n">
-        <v>46279.25</v>
+        <v>46278.91666666666</v>
       </c>
       <c r="H101" s="3" t="n">
-        <v>46279.41666666666</v>
+        <v>46279.08333333334</v>
       </c>
       <c r="I101" s="3" t="n">
-        <v>46279.95833333334</v>
+        <v>46279.625</v>
       </c>
     </row>
     <row r="102">
@@ -6708,13 +6708,13 @@
         </is>
       </c>
       <c r="G102" s="3" t="n">
-        <v>46285.54166666666</v>
+        <v>46285.20833333334</v>
       </c>
       <c r="H102" s="3" t="n">
-        <v>46285.58333333334</v>
+        <v>46285.25</v>
       </c>
       <c r="I102" s="3" t="n">
-        <v>46286.66666666666</v>
+        <v>46286.33333333334</v>
       </c>
     </row>
     <row r="103">
@@ -6749,13 +6749,13 @@
         </is>
       </c>
       <c r="G103" s="3" t="n">
-        <v>46286.79166666666</v>
+        <v>46286.45833333334</v>
       </c>
       <c r="H103" s="3" t="n">
-        <v>46286.83333333334</v>
+        <v>46286.5</v>
       </c>
       <c r="I103" s="3" t="n">
-        <v>46287.08333333334</v>
+        <v>46286.75</v>
       </c>
     </row>
     <row r="104">
@@ -6790,13 +6790,13 @@
         </is>
       </c>
       <c r="G104" s="3" t="n">
-        <v>46287.45833333334</v>
+        <v>46287.125</v>
       </c>
       <c r="H104" s="3" t="n">
+        <v>46287.1875</v>
+      </c>
+      <c r="I104" s="3" t="n">
         <v>46287.52083333334</v>
-      </c>
-      <c r="I104" s="3" t="n">
-        <v>46287.85416666666</v>
       </c>
     </row>
     <row r="105">
@@ -6831,13 +6831,13 @@
         </is>
       </c>
       <c r="G105" s="3" t="n">
-        <v>46293.08333333334</v>
+        <v>46292.75</v>
       </c>
       <c r="H105" s="3" t="n">
-        <v>46293.25</v>
+        <v>46292.91666666666</v>
       </c>
       <c r="I105" s="3" t="n">
-        <v>46293.875</v>
+        <v>46293.54166666666</v>
       </c>
     </row>
     <row r="106">
@@ -6872,13 +6872,13 @@
         </is>
       </c>
       <c r="G106" s="3" t="n">
-        <v>46295.625</v>
+        <v>46295.29166666666</v>
       </c>
       <c r="H106" s="3" t="n">
-        <v>46295.66666666666</v>
+        <v>46295.33333333334</v>
       </c>
       <c r="I106" s="3" t="n">
-        <v>46295.91666666666</v>
+        <v>46295.58333333334</v>
       </c>
     </row>
     <row r="107">
@@ -6913,13 +6913,13 @@
         </is>
       </c>
       <c r="G107" s="3" t="n">
-        <v>46296.04166666666</v>
+        <v>46295.70833333334</v>
       </c>
       <c r="H107" s="3" t="n">
-        <v>46296.16666666666</v>
+        <v>46295.83333333334</v>
       </c>
       <c r="I107" s="3" t="n">
-        <v>46297.66666666666</v>
+        <v>46297.33333333334</v>
       </c>
     </row>
     <row r="108">
@@ -6954,13 +6954,13 @@
         </is>
       </c>
       <c r="G108" s="3" t="n">
-        <v>46297.875</v>
+        <v>46297.54166666666</v>
       </c>
       <c r="H108" s="3" t="n">
-        <v>46297.91666666666</v>
+        <v>46297.58333333334</v>
       </c>
       <c r="I108" s="3" t="n">
-        <v>46298.33333333334</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="109">
@@ -6995,13 +6995,13 @@
         </is>
       </c>
       <c r="G109" s="3" t="n">
-        <v>46299.91666666666</v>
+        <v>46299.58333333334</v>
       </c>
       <c r="H109" s="3" t="n">
-        <v>46300.08333333334</v>
+        <v>46299.75</v>
       </c>
       <c r="I109" s="3" t="n">
-        <v>46300.625</v>
+        <v>46300.29166666666</v>
       </c>
     </row>
     <row r="110">
@@ -7036,13 +7036,13 @@
         </is>
       </c>
       <c r="G110" s="3" t="n">
-        <v>46305.91666666666</v>
+        <v>46305.58333333334</v>
       </c>
       <c r="H110" s="3" t="n">
-        <v>46305.95833333334</v>
+        <v>46305.625</v>
       </c>
       <c r="I110" s="3" t="n">
-        <v>46307.04166666666</v>
+        <v>46306.70833333334</v>
       </c>
     </row>
     <row r="111">
@@ -7077,13 +7077,13 @@
         </is>
       </c>
       <c r="G111" s="3" t="n">
-        <v>46307.16666666666</v>
+        <v>46306.83333333334</v>
       </c>
       <c r="H111" s="3" t="n">
-        <v>46307.20833333334</v>
+        <v>46306.875</v>
       </c>
       <c r="I111" s="3" t="n">
-        <v>46307.45833333334</v>
+        <v>46307.125</v>
       </c>
     </row>
     <row r="112">
@@ -7118,13 +7118,13 @@
         </is>
       </c>
       <c r="G112" s="3" t="n">
-        <v>46307.875</v>
+        <v>46307.54166666666</v>
       </c>
       <c r="H112" s="3" t="n">
+        <v>46307.625</v>
+      </c>
+      <c r="I112" s="3" t="n">
         <v>46307.95833333334</v>
-      </c>
-      <c r="I112" s="3" t="n">
-        <v>46308.29166666666</v>
       </c>
     </row>
     <row r="113">
@@ -7159,13 +7159,13 @@
         </is>
       </c>
       <c r="G113" s="3" t="n">
-        <v>46313.29166666666</v>
+        <v>46312.95833333334</v>
       </c>
       <c r="H113" s="3" t="n">
-        <v>46313.45833333334</v>
+        <v>46313.125</v>
       </c>
       <c r="I113" s="3" t="n">
-        <v>46314.08333333334</v>
+        <v>46313.75</v>
       </c>
     </row>
     <row r="114">
@@ -7200,13 +7200,13 @@
         </is>
       </c>
       <c r="G114" s="3" t="n">
-        <v>46315.875</v>
+        <v>46315.54166666666</v>
       </c>
       <c r="H114" s="3" t="n">
-        <v>46315.91666666666</v>
+        <v>46315.58333333334</v>
       </c>
       <c r="I114" s="3" t="n">
-        <v>46316.16666666666</v>
+        <v>46315.83333333334</v>
       </c>
     </row>
     <row r="115">
@@ -7241,13 +7241,13 @@
         </is>
       </c>
       <c r="G115" s="3" t="n">
-        <v>46316.45833333334</v>
+        <v>46316.125</v>
       </c>
       <c r="H115" s="3" t="n">
-        <v>46316.58333333334</v>
+        <v>46316.25</v>
       </c>
       <c r="I115" s="3" t="n">
-        <v>46318.08333333334</v>
+        <v>46317.75</v>
       </c>
     </row>
     <row r="116">
@@ -7282,13 +7282,13 @@
         </is>
       </c>
       <c r="G116" s="3" t="n">
-        <v>46318.29166666666</v>
+        <v>46317.95833333334</v>
       </c>
       <c r="H116" s="3" t="n">
-        <v>46318.33333333334</v>
+        <v>46318</v>
       </c>
       <c r="I116" s="3" t="n">
-        <v>46318.75</v>
+        <v>46318.41666666666</v>
       </c>
     </row>
     <row r="117">
@@ -7323,13 +7323,13 @@
         </is>
       </c>
       <c r="G117" s="3" t="n">
-        <v>46320.33333333334</v>
+        <v>46320</v>
       </c>
       <c r="H117" s="3" t="n">
-        <v>46320.5</v>
+        <v>46320.16666666666</v>
       </c>
       <c r="I117" s="3" t="n">
-        <v>46321.04166666666</v>
+        <v>46320.70833333334</v>
       </c>
     </row>
     <row r="118">
@@ -7364,13 +7364,13 @@
         </is>
       </c>
       <c r="G118" s="3" t="n">
-        <v>46326.20833333334</v>
+        <v>46325.875</v>
       </c>
       <c r="H118" s="3" t="n">
-        <v>46326.25</v>
+        <v>46325.91666666666</v>
       </c>
       <c r="I118" s="3" t="n">
-        <v>46327.33333333334</v>
+        <v>46327</v>
       </c>
     </row>
     <row r="119">
@@ -7405,13 +7405,13 @@
         </is>
       </c>
       <c r="G119" s="3" t="n">
-        <v>46327.45833333334</v>
+        <v>46327.125</v>
       </c>
       <c r="H119" s="3" t="n">
-        <v>46327.5</v>
+        <v>46327.16666666666</v>
       </c>
       <c r="I119" s="3" t="n">
-        <v>46327.75</v>
+        <v>46327.41666666666</v>
       </c>
     </row>
     <row r="120">
@@ -7446,13 +7446,13 @@
         </is>
       </c>
       <c r="G120" s="3" t="n">
-        <v>46328.16666666666</v>
+        <v>46327.83333333334</v>
       </c>
       <c r="H120" s="3" t="n">
+        <v>46327.91666666666</v>
+      </c>
+      <c r="I120" s="3" t="n">
         <v>46328.25</v>
-      </c>
-      <c r="I120" s="3" t="n">
-        <v>46328.58333333334</v>
       </c>
     </row>
     <row r="121">
@@ -7487,13 +7487,13 @@
         </is>
       </c>
       <c r="G121" s="3" t="n">
-        <v>46333.58333333334</v>
+        <v>46333.25</v>
       </c>
       <c r="H121" s="3" t="n">
-        <v>46333.75</v>
+        <v>46333.41666666666</v>
       </c>
       <c r="I121" s="3" t="n">
-        <v>46334.375</v>
+        <v>46334.04166666666</v>
       </c>
     </row>
     <row r="122">
@@ -7528,13 +7528,13 @@
         </is>
       </c>
       <c r="G122" s="3" t="n">
-        <v>46336.16666666666</v>
+        <v>46335.83333333334</v>
       </c>
       <c r="H122" s="3" t="n">
-        <v>46336.20833333334</v>
+        <v>46335.875</v>
       </c>
       <c r="I122" s="3" t="n">
-        <v>46336.45833333334</v>
+        <v>46336.125</v>
       </c>
     </row>
     <row r="123">
@@ -7569,13 +7569,13 @@
         </is>
       </c>
       <c r="G123" s="3" t="n">
-        <v>46336.75</v>
+        <v>46336.41666666666</v>
       </c>
       <c r="H123" s="3" t="n">
-        <v>46336.875</v>
+        <v>46336.54166666666</v>
       </c>
       <c r="I123" s="3" t="n">
-        <v>46338.375</v>
+        <v>46338.04166666666</v>
       </c>
     </row>
     <row r="124">
@@ -28499,15 +28499,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
@@ -28535,12 +28535,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>New ETA (patched: _test_kmbk_partial.xlsx (KMTC BANGKOK))</t>
+          <t>New ETA (9-10-1030-SKED.xls)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -28551,978 +28551,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>2610S</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>46274.16666666666</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>46274.5</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>2610N</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>46274.75</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>46275.08333333334</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>2610N</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>46274.75</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>46275.08333333334</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2610N</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>46276.83333333334</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>46277.16666666666</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>KRKAN</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2610N</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>46278.91666666666</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>46279.25</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2611S</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>46285.20833333334</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>46285.54166666666</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>KRUSN</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>KRUSN</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2611S</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>46286.45833333334</v>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>46286.79166666666</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>KRKAN</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2611S</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>46287.125</v>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>46287.45833333334</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2611S</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>46292.75</v>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>46293.08333333334</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2611S</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>46295.29166666666</v>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>46295.625</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2611N</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>46295.70833333334</v>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>46296.04166666666</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2611N</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>46297.54166666666</v>
-      </c>
-      <c r="F13" s="3" t="n">
-        <v>46297.875</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>KRKAN</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2611N</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>46299.58333333334</v>
-      </c>
-      <c r="F14" s="3" t="n">
-        <v>46299.91666666666</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2612S</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>46305.58333333334</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>46305.91666666666</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>KRUSN</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>KRUSN</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2612S</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>46306.83333333334</v>
-      </c>
-      <c r="F16" s="3" t="n">
-        <v>46307.16666666666</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>KRKAN</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>2612S</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>46307.54166666666</v>
-      </c>
-      <c r="F17" s="3" t="n">
-        <v>46307.875</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2612S</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>46312.95833333334</v>
-      </c>
-      <c r="F18" s="3" t="n">
-        <v>46313.29166666666</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>2612S</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>46315.54166666666</v>
-      </c>
-      <c r="F19" s="3" t="n">
-        <v>46315.875</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>2612N</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="n">
-        <v>46316.125</v>
-      </c>
-      <c r="F20" s="3" t="n">
-        <v>46316.45833333334</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>2612N</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="n">
-        <v>46317.95833333334</v>
-      </c>
-      <c r="F21" s="3" t="n">
-        <v>46318.29166666666</v>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>KRKAN</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>2612N</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="n">
-        <v>46320</v>
-      </c>
-      <c r="F22" s="3" t="n">
-        <v>46320.33333333334</v>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>2613S</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>46325.875</v>
-      </c>
-      <c r="F23" s="3" t="n">
-        <v>46326.20833333334</v>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>KRUSN</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>KRUSN</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>2613S</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="n">
-        <v>46327.125</v>
-      </c>
-      <c r="F24" s="3" t="n">
-        <v>46327.45833333334</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>KRKAN</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>2613S</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="n">
-        <v>46327.83333333334</v>
-      </c>
-      <c r="F25" s="3" t="n">
-        <v>46328.16666666666</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>2613S</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>46333.25</v>
-      </c>
-      <c r="F26" s="3" t="n">
-        <v>46333.58333333334</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>2613S</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>46335.83333333334</v>
-      </c>
-      <c r="F27" s="3" t="n">
-        <v>46336.16666666666</v>
-      </c>
-      <c r="G27" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>2613N</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="n">
-        <v>46336.41666666666</v>
-      </c>
-      <c r="F28" s="3" t="n">
-        <v>46336.75</v>
-      </c>
-      <c r="G28" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>Delay</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add live real-time clock to dashboard toolbar
Adds a ticking date/time readout (day, Buddhist-era date, HH:MM:SS) next
to the data-source status line, filling the empty space in that row.
Re-renders Vessel Schedule.html/.xlsx from the existing sked_current.xlsx
snapshot (data unchanged, template only) without disturbing sked_prev.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1443,20 +1443,22 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>transit</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>KRKAN -&gt; KRPUS</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v/>
+          <t>KRPUS (PUS05)</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2611S</t>
+        </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>In transit, ETA 2026-09-11T12:00:00</t>
+          <t>Alongside, departs to VNSGN ~2026-09-13T07:00:00</t>
         </is>
       </c>
       <c r="I16" s="3" t="n">

</xml_diff>

<commit_message>
Fix header overflow on narrow mobile screens
The logo had flex-shrink:0 inside the flex header, so on real phone
widths (~360-420px) it refused to shrink and forced the "TERMINAL OPS"
eyebrow / "Vessel Schedule" title text into an overflowing sliver,
which made the whole page render squeezed/cut off (confirmed via
scrollWidth > clientWidth on .brand-block).

Fix: let the logo shrink, and below 480px stack logo above the title
text instead of side-by-side, so both always have their own full-width
row. Also adds html/body overflow-x:hidden as a safety net against any
future overflow causing the same zoomed-out effect. Verified no
horizontal overflow at 360/375/412px widths.

Re-renders from the existing sked_current.xlsx snapshot (data unchanged)
without touching sked_prev.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -553,20 +553,22 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>nodata</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v/>
+          <t>KRPUS (PUSH4)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2614S</t>
+        </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>No data in window</t>
+          <t>Alongside, departs to KRUSN ~2026-09-13T00:00:00</t>
         </is>
       </c>
       <c r="I2" s="3" t="n">
@@ -871,12 +873,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>nodata</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>THLCH -&gt; VNSGN</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
@@ -884,7 +886,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>No data in window</t>
+          <t>In transit, ETA 2026-09-13T22:00:00</t>
         </is>
       </c>
       <c r="I7" s="3" t="n">
@@ -901,7 +903,7 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>46276.83333333334</v>
+        <v>46295.29166666666</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
@@ -910,7 +912,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2611S</t>
         </is>
       </c>
     </row>
@@ -937,20 +939,22 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>nodata</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v/>
+          <t>KRINC (INC03)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2610S</t>
+        </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>No data in window</t>
+          <t>Alongside, departs to CNTAO ~2026-09-12T18:00:00</t>
         </is>
       </c>
       <c r="I8" s="3" t="n">
@@ -1069,20 +1073,22 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>nodata</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v/>
+          <t>KRINC (INC08)</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2607S</t>
+        </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>No data in window</t>
+          <t>Alongside, departs to KRPUS ~2026-09-12T18:00:00</t>
         </is>
       </c>
       <c r="I10" s="3" t="n"/>
@@ -1261,20 +1267,22 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>nodata</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v/>
+          <t>VNSGN (SGN03)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2607N</t>
+        </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>No data in window</t>
+          <t>Alongside, departs to HKHKG ~2026-09-13T16:00:00</t>
         </is>
       </c>
       <c r="I13" s="3" t="n"/>
@@ -1709,22 +1717,20 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>THBKK (BKK02)</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>2609N</t>
-        </is>
+          <t>THLCH -&gt; VNSGN</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v/>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to THLCH ~2026-09-11T18:00:00</t>
+          <t>In transit, ETA 2026-09-13T22:00:00</t>
         </is>
       </c>
       <c r="I20" s="3" t="n"/>
@@ -1735,16 +1741,16 @@
         <v/>
       </c>
       <c r="L20" s="3" t="n">
-        <v>46276.91666666666</v>
+        <v>46305.16666666666</v>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>LCH01</t>
+          <t>LCH06</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2610N</t>
         </is>
       </c>
     </row>
@@ -1837,22 +1843,20 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>KRUSN (USN03)</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>2610S</t>
-        </is>
+          <t>KRUSN -&gt; VNSGN</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v/>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to VNSGN ~2026-09-11T22:00:00</t>
+          <t>In transit, ETA 2026-09-17T01:00:00</t>
         </is>
       </c>
       <c r="I22" s="3" t="n">
@@ -2223,22 +2227,20 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>CNXMN (XMN01)</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>2610N</t>
-        </is>
+          <t>CNXMN -&gt; KRPUS</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v/>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to KRPUS ~2026-09-11T23:30:00</t>
+          <t>In transit, ETA 2026-09-14T08:00:00</t>
         </is>
       </c>
       <c r="I28" s="3" t="n">

</xml_diff>